<commit_message>
DEV: Fixed formatting violations. Fixed missing private functions in Copy-IRTFunction.
</commit_message>
<xml_diff>
--- a/Source/Data/UALAllOperations.xlsx
+++ b/Source/Data/UALAllOperations.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2368" uniqueCount="2368">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2369" uniqueCount="2369">
   <si>
     <t>Risk</t>
   </si>
@@ -7124,6 +7124,9 @@
   </si>
   <si>
     <t>Add delegated permission grant.</t>
+  </si>
+  <si>
+    <t>CallParticipantDetail</t>
   </si>
 </sst>
 </file>
@@ -7890,8 +7893,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{43428C69-B5D7-486D-BCF0-3E3383702390}" name="Table1" displayName="Table1" ref="A1:G847" totalsRowShown="0">
-  <autoFilter ref="A1:G844" xr:uid="{43428C69-B5D7-486D-BCF0-3E3383702390}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{43428C69-B5D7-486D-BCF0-3E3383702390}" name="Table1" displayName="Table1" ref="A1:G848" totalsRowShown="0">
+  <autoFilter ref="A1:G847" xr:uid="{43428C69-B5D7-486D-BCF0-3E3383702390}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G835">
     <sortCondition ref="D2:D835"/>
   </sortState>
@@ -8225,7 +8228,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{207B3246-3E1F-4883-B5B7-F0312ED8EA41}">
-  <dimension ref="A1:G847"/>
+  <dimension ref="A1:G848"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" bestFit="1" width="8.140625" customWidth="1"/>
@@ -18038,6 +18041,17 @@
       </c>
       <c r="D847" s="0" t="s">
         <v>2367</v>
+      </c>
+    </row>
+    <row r="848">
+      <c r="B848" s="0" t="s">
+        <v>1152</v>
+      </c>
+      <c r="C848" s="0" t="s">
+        <v>1152</v>
+      </c>
+      <c r="D848" s="0" t="s">
+        <v>2368</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
FEATURE: Added ResultLimit param to stop query when there are excessive results. Added chunking for queries over 6 months.
</commit_message>
<xml_diff>
--- a/Source/Data/UALAllOperations.xlsx
+++ b/Source/Data/UALAllOperations.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2375" uniqueCount="2375">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2376" uniqueCount="2376">
   <si>
     <t>Risk</t>
   </si>
@@ -7145,6 +7145,9 @@
   </si>
   <si>
     <t>Delete application.</t>
+  </si>
+  <si>
+    <t>Remove-StoreMailbox</t>
   </si>
 </sst>
 </file>
@@ -7911,8 +7914,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{43428C69-B5D7-486D-BCF0-3E3383702390}" name="Table1" displayName="Table1" ref="A1:G855" totalsRowShown="0">
-  <autoFilter ref="A1:G848" xr:uid="{43428C69-B5D7-486D-BCF0-3E3383702390}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{43428C69-B5D7-486D-BCF0-3E3383702390}" name="Table1" displayName="Table1" ref="A1:G856" totalsRowShown="0">
+  <autoFilter ref="A1:G855" xr:uid="{43428C69-B5D7-486D-BCF0-3E3383702390}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G835">
     <sortCondition ref="D2:D835"/>
   </sortState>
@@ -8246,7 +8249,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{207B3246-3E1F-4883-B5B7-F0312ED8EA41}">
-  <dimension ref="A1:G855"/>
+  <dimension ref="A1:G856"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" bestFit="1" width="8.140625" customWidth="1"/>
@@ -18147,6 +18150,17 @@
       </c>
       <c r="D855" s="0" t="s">
         <v>2374</v>
+      </c>
+    </row>
+    <row r="856">
+      <c r="B856" s="0" t="s">
+        <v>213</v>
+      </c>
+      <c r="C856" s="0" t="s">
+        <v>594</v>
+      </c>
+      <c r="D856" s="0" t="s">
+        <v>2375</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: updated alloperations spreadsheet.
</commit_message>
<xml_diff>
--- a/Source/Data/UALAllOperations.xlsx
+++ b/Source/Data/UALAllOperations.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2376" uniqueCount="2376">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2387" uniqueCount="2387">
   <si>
     <t>Risk</t>
   </si>
@@ -7148,6 +7148,39 @@
   </si>
   <si>
     <t>Remove-StoreMailbox</t>
+  </si>
+  <si>
+    <t>ModifyFolderPermissions</t>
+  </si>
+  <si>
+    <t>MessageReadReceiptReceived</t>
+  </si>
+  <si>
+    <t>FileVersionsAllDeleted</t>
+  </si>
+  <si>
+    <t>FeatureActivated</t>
+  </si>
+  <si>
+    <t>SPOTenantCmdlets</t>
+  </si>
+  <si>
+    <t>MicrosoftTodo</t>
+  </si>
+  <si>
+    <t>MicrosoftTodoAudit</t>
+  </si>
+  <si>
+    <t>Copilot</t>
+  </si>
+  <si>
+    <t>Remove app role assignment from user.</t>
+  </si>
+  <si>
+    <t>Add policy to service principal.</t>
+  </si>
+  <si>
+    <t>Add device.</t>
   </si>
 </sst>
 </file>
@@ -7914,8 +7947,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{43428C69-B5D7-486D-BCF0-3E3383702390}" name="Table1" displayName="Table1" ref="A1:G856" totalsRowShown="0">
-  <autoFilter ref="A1:G855" xr:uid="{43428C69-B5D7-486D-BCF0-3E3383702390}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{43428C69-B5D7-486D-BCF0-3E3383702390}" name="Table1" displayName="Table1" ref="A1:G886" totalsRowShown="0">
+  <autoFilter ref="A1:G883" xr:uid="{43428C69-B5D7-486D-BCF0-3E3383702390}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G835">
     <sortCondition ref="D2:D835"/>
   </sortState>
@@ -8249,7 +8282,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{207B3246-3E1F-4883-B5B7-F0312ED8EA41}">
-  <dimension ref="A1:G856"/>
+  <dimension ref="A1:G886"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" bestFit="1" width="8.140625" customWidth="1"/>
@@ -18161,6 +18194,336 @@
       </c>
       <c r="D856" s="0" t="s">
         <v>2375</v>
+      </c>
+    </row>
+    <row r="857">
+      <c r="B857" s="0" t="s">
+        <v>1152</v>
+      </c>
+      <c r="C857" s="0" t="s">
+        <v>1152</v>
+      </c>
+      <c r="D857" s="0" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="858">
+      <c r="B858" s="0" t="s">
+        <v>1152</v>
+      </c>
+      <c r="C858" s="0" t="s">
+        <v>1152</v>
+      </c>
+      <c r="D858" s="0" t="s">
+        <v>2122</v>
+      </c>
+    </row>
+    <row r="859">
+      <c r="B859" s="0" t="s">
+        <v>213</v>
+      </c>
+      <c r="C859" s="0" t="s">
+        <v>456</v>
+      </c>
+      <c r="D859" s="0" t="s">
+        <v>2376</v>
+      </c>
+    </row>
+    <row r="860">
+      <c r="B860" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="C860" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="D860" s="0" t="s">
+        <v>1845</v>
+      </c>
+    </row>
+    <row r="861">
+      <c r="B861" s="0" t="s">
+        <v>1152</v>
+      </c>
+      <c r="C861" s="0" t="s">
+        <v>1152</v>
+      </c>
+      <c r="D861" s="0" t="s">
+        <v>2377</v>
+      </c>
+    </row>
+    <row r="862">
+      <c r="B862" s="0" t="s">
+        <v>377</v>
+      </c>
+      <c r="C862" s="0" t="s">
+        <v>737</v>
+      </c>
+      <c r="D862" s="0" t="s">
+        <v>768</v>
+      </c>
+    </row>
+    <row r="863">
+      <c r="B863" s="0" t="s">
+        <v>377</v>
+      </c>
+      <c r="C863" s="0" t="s">
+        <v>737</v>
+      </c>
+      <c r="D863" s="0" t="s">
+        <v>2378</v>
+      </c>
+    </row>
+    <row r="864">
+      <c r="B864" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="C864" s="0" t="s">
+        <v>377</v>
+      </c>
+      <c r="D864" s="0" t="s">
+        <v>2379</v>
+      </c>
+    </row>
+    <row r="865">
+      <c r="B865" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="C865" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="D865" s="0" t="s">
+        <v>1875</v>
+      </c>
+    </row>
+    <row r="866">
+      <c r="B866" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="C866" s="0" t="s">
+        <v>737</v>
+      </c>
+      <c r="D866" s="0" t="s">
+        <v>854</v>
+      </c>
+    </row>
+    <row r="867">
+      <c r="B867" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="C867" s="0" t="s">
+        <v>737</v>
+      </c>
+      <c r="D867" s="0" t="s">
+        <v>842</v>
+      </c>
+    </row>
+    <row r="868">
+      <c r="B868" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="C868" s="0" t="s">
+        <v>377</v>
+      </c>
+      <c r="D868" s="0" t="s">
+        <v>1904</v>
+      </c>
+    </row>
+    <row r="869">
+      <c r="B869" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="C869" s="0" t="s">
+        <v>377</v>
+      </c>
+      <c r="D869" s="0" t="s">
+        <v>1866</v>
+      </c>
+    </row>
+    <row r="870">
+      <c r="B870" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="C870" s="0" t="s">
+        <v>377</v>
+      </c>
+      <c r="D870" s="0" t="s">
+        <v>2380</v>
+      </c>
+    </row>
+    <row r="871">
+      <c r="B871" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="C871" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="D871" s="0" t="s">
+        <v>1898</v>
+      </c>
+    </row>
+    <row r="872">
+      <c r="B872" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="C872" s="0" t="s">
+        <v>377</v>
+      </c>
+      <c r="D872" s="0" t="s">
+        <v>1901</v>
+      </c>
+    </row>
+    <row r="873">
+      <c r="B873" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="C873" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="D873" s="0" t="s">
+        <v>1895</v>
+      </c>
+    </row>
+    <row r="874">
+      <c r="B874" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="C874" s="0" t="s">
+        <v>377</v>
+      </c>
+      <c r="D874" s="0" t="s">
+        <v>1949</v>
+      </c>
+    </row>
+    <row r="875">
+      <c r="B875" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="C875" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="D875" s="0" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="876">
+      <c r="B876" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="C876" s="0" t="s">
+        <v>377</v>
+      </c>
+      <c r="D876" s="0" t="s">
+        <v>1317</v>
+      </c>
+    </row>
+    <row r="877">
+      <c r="B877" s="0" t="s">
+        <v>213</v>
+      </c>
+      <c r="C877" s="0" t="s">
+        <v>961</v>
+      </c>
+      <c r="D877" s="0" t="s">
+        <v>1223</v>
+      </c>
+    </row>
+    <row r="878">
+      <c r="B878" s="0" t="s">
+        <v>2381</v>
+      </c>
+      <c r="C878" s="0" t="s">
+        <v>2382</v>
+      </c>
+      <c r="D878" s="0" t="s">
+        <v>2066</v>
+      </c>
+    </row>
+    <row r="879">
+      <c r="B879" s="0" t="s">
+        <v>2383</v>
+      </c>
+      <c r="C879" s="0" t="s">
+        <v>450</v>
+      </c>
+      <c r="D879" s="0" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="880">
+      <c r="B880" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="C880" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="D880" s="0" t="s">
+        <v>2384</v>
+      </c>
+    </row>
+    <row r="881">
+      <c r="B881" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="C881" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="D881" s="0" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="882">
+      <c r="B882" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="C882" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="D882" s="0" t="s">
+        <v>2385</v>
+      </c>
+    </row>
+    <row r="883">
+      <c r="B883" s="0" t="s">
+        <v>1152</v>
+      </c>
+      <c r="C883" s="0" t="s">
+        <v>1152</v>
+      </c>
+      <c r="D883" s="0" t="s">
+        <v>1165</v>
+      </c>
+    </row>
+    <row r="884">
+      <c r="B884" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="C884" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="D884" s="0" t="s">
+        <v>2386</v>
+      </c>
+    </row>
+    <row r="885">
+      <c r="B885" s="0" t="s">
+        <v>377</v>
+      </c>
+      <c r="C885" s="0" t="s">
+        <v>737</v>
+      </c>
+      <c r="D885" s="0" t="s">
+        <v>777</v>
+      </c>
+    </row>
+    <row r="886">
+      <c r="B886" s="0" t="s">
+        <v>377</v>
+      </c>
+      <c r="C886" s="0" t="s">
+        <v>737</v>
+      </c>
+      <c r="D886" s="0" t="s">
+        <v>774</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): add MicrosoftTeams MemberRoleChanged to the operations sheet
Appended by Build-AllOperationSheet during live testing, which adds any
operation it meets that is missing from the reference sheet. Risk and Summary
are blank pending classification.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Source/Data/UALAllOperations.xlsx
+++ b/Source/Data/UALAllOperations.xlsx
@@ -7902,8 +7902,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{43428C69-B5D7-486D-BCF0-3E3383702390}" name="Table1" displayName="Table1" ref="A1:G952" totalsRowShown="0">
-  <autoFilter ref="A1:G947" xr:uid="{43428C69-B5D7-486D-BCF0-3E3383702390}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{43428C69-B5D7-486D-BCF0-3E3383702390}" name="Table1" displayName="Table1" ref="A1:G953" totalsRowShown="0">
+  <autoFilter ref="A1:G952" xr:uid="{43428C69-B5D7-486D-BCF0-3E3383702390}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G835">
     <sortCondition ref="D2:D835"/>
   </sortState>
@@ -8237,7 +8237,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{207B3246-3E1F-4883-B5B7-F0312ED8EA41}">
-  <dimension ref="A1:G952"/>
+  <dimension ref="A1:G953"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" bestFit="1" width="8.140625" customWidth="1"/>
@@ -19208,6 +19208,17 @@
       </c>
       <c r="D952" s="0" t="s">
         <v>857</v>
+      </c>
+    </row>
+    <row r="953">
+      <c r="B953" s="0" t="s">
+        <v>1152</v>
+      </c>
+      <c r="C953" s="0" t="s">
+        <v>1152</v>
+      </c>
+      <c r="D953" s="0" t="s">
+        <v>1162</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): add the AuditSearch operations to the operations sheet
Add AuditSearchCreated and AuditSearchCompleted, SecurityComplianceCenter
operations under the AuditSearch record type. Neither row has a friendly
name, description, or risk yet.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Source/Data/UALAllOperations.xlsx
+++ b/Source/Data/UALAllOperations.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2432" uniqueCount="2432">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2433" uniqueCount="2433">
   <si>
     <t>Risk</t>
   </si>
@@ -7316,6 +7316,9 @@
   </si>
   <si>
     <t>AccessRequestApproved</t>
+  </si>
+  <si>
+    <t>AuditSearch</t>
   </si>
 </sst>
 </file>
@@ -7902,8 +7905,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{43428C69-B5D7-486D-BCF0-3E3383702390}" name="Table1" displayName="Table1" ref="A1:G953" totalsRowShown="0">
-  <autoFilter ref="A1:G952" xr:uid="{43428C69-B5D7-486D-BCF0-3E3383702390}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{43428C69-B5D7-486D-BCF0-3E3383702390}" name="Table1" displayName="Table1" ref="A1:G955" totalsRowShown="0">
+  <autoFilter ref="A1:G953" xr:uid="{43428C69-B5D7-486D-BCF0-3E3383702390}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G835">
     <sortCondition ref="D2:D835"/>
   </sortState>
@@ -8237,7 +8240,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{207B3246-3E1F-4883-B5B7-F0312ED8EA41}">
-  <dimension ref="A1:G953"/>
+  <dimension ref="A1:G955"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" bestFit="1" width="8.140625" customWidth="1"/>
@@ -19219,6 +19222,28 @@
       </c>
       <c r="D953" s="0" t="s">
         <v>1162</v>
+      </c>
+    </row>
+    <row r="954">
+      <c r="B954" s="0" t="s">
+        <v>117</v>
+      </c>
+      <c r="C954" s="0" t="s">
+        <v>2432</v>
+      </c>
+      <c r="D954" s="0" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="955">
+      <c r="B955" s="0" t="s">
+        <v>117</v>
+      </c>
+      <c r="C955" s="0" t="s">
+        <v>2432</v>
+      </c>
+      <c r="D955" s="0" t="s">
+        <v>231</v>
       </c>
     </row>
   </sheetData>

</xml_diff>